<commit_message>
Updated buy sell signals
</commit_message>
<xml_diff>
--- a/MCX_Trading_Platform_Data.xlsx
+++ b/MCX_Trading_Platform_Data.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,6 +437,72 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.179716412037037</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.1797401388888889</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.1797636574074074</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.1797874074074074</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0.1798110185185185</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0.1798346944212963</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated code auto trade
</commit_message>
<xml_diff>
--- a/MCX_Trading_Platform_Data.xlsx
+++ b/MCX_Trading_Platform_Data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,7 +442,7 @@
         <v>46033</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.179716412037037</v>
+        <v>0.7808441319444445</v>
       </c>
       <c r="C2" t="n">
         <v>-1.5</v>
@@ -453,7 +453,7 @@
         <v>46033</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.1797401388888889</v>
+        <v>0.7808679976851851</v>
       </c>
       <c r="C3" t="n">
         <v>-1.5</v>
@@ -464,7 +464,7 @@
         <v>46033</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.1797636574074074</v>
+        <v>0.7808914930555555</v>
       </c>
       <c r="C4" t="n">
         <v>-1.5</v>
@@ -475,7 +475,7 @@
         <v>46033</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.1797874074074074</v>
+        <v>0.7809153935185185</v>
       </c>
       <c r="C5" t="n">
         <v>-1.5</v>
@@ -486,7 +486,7 @@
         <v>46033</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.1798110185185185</v>
+        <v>0.7809386921296296</v>
       </c>
       <c r="C6" t="n">
         <v>-1.5</v>
@@ -497,9 +497,20 @@
         <v>46033</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.1798346944212963</v>
+        <v>0.7809624768518518</v>
       </c>
       <c r="C7" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46033</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0.780986313125</v>
+      </c>
+      <c r="C8" t="n">
         <v>-1.5</v>
       </c>
     </row>

</xml_diff>